<commit_message>
raw data pulled out of main model script.
</commit_message>
<xml_diff>
--- a/data-raw/Carer disutilities.xlsx
+++ b/data-raw/Carer disutilities.xlsx
@@ -666,8 +666,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACE3D2A8E3060445845CB33F649944D9" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7c8efc5d897a5a54c153d61be50fc1e0">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a4e98822-f433-4c96-8830-5cb2d7491f7d" xmlns:ns3="adc125f1-7df9-46f4-a9a7-022dd426a2bb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7c927ce20f93a00fedc297caf603d12c" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACE3D2A8E3060445845CB33F649944D9" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1dd74ed78a59e353fa0bdc00cb9d4ef2">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a4e98822-f433-4c96-8830-5cb2d7491f7d" xmlns:ns3="adc125f1-7df9-46f4-a9a7-022dd426a2bb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29b19980e720fd97176dcdbc89cda831" ns2:_="" ns3:_="">
     <xsd:import namespace="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
     <xsd:import namespace="adc125f1-7df9-46f4-a9a7-022dd426a2bb"/>
     <xsd:element name="properties">
@@ -885,23 +885,18 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a4e98822-f433-4c96-8830-5cb2d7491f7d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0C5D4B03-6E00-478A-9671-5FE48F2C6CE8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
-    <ds:schemaRef ds:uri="adc125f1-7df9-46f4-a9a7-022dd426a2bb"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F0B826-5EFE-4577-B049-981EAE9E4CA2}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -910,4 +905,8 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32834C50-F458-4BC1-999D-E35548F4265A}"/>
 </file>
</xml_diff>

<commit_message>
Scripts and data post comments
</commit_message>
<xml_diff>
--- a/data-raw/Carer disutilities.xlsx
+++ b/data-raw/Carer disutilities.xlsx
@@ -1,21 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="123820"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob.sharepoint.com/teams/grp-Bristol_TAG-MTA-MS/Shared Documents/MTA-MS/Working Folder_HE/MS Models/Git Repo/MS-MTA/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\po22525\University of Bristol\grp-Bristol TAG - MTA-MS - MTA-MS\Working Folder_HE\MS Models\Git Repo\MS-MTA\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_4232EF2381E847C1BB976A383DF301233CDD491F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B8F52FA-6919-4699-B46B-9752F03F3A96}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CDB371A-1B3B-471D-8F3B-FF3061DDA828}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32775" yWindow="-15135" windowWidth="17280" windowHeight="11730" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Acaster" sheetId="1" r:id="rId1"/>
+    <sheet name="TA127" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -71,6 +85,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.000"/>
+  </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -150,7 +167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -161,6 +178,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -665,7 +683,160 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E6C296D-3E9C-4769-B446-B20A29C524FE}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" t="str">
+        <f>Acaster!A1</f>
+        <v>State</v>
+      </c>
+      <c r="B1" t="str">
+        <f>Acaster!B1</f>
+        <v>Mean</v>
+      </c>
+      <c r="C1" t="str">
+        <f>Acaster!C1</f>
+        <v xml:space="preserve">SE </v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="str">
+        <f>Acaster!A2</f>
+        <v>EDSS 0</v>
+      </c>
+      <c r="B2" s="4">
+        <v>0</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="str">
+        <f>Acaster!A3</f>
+        <v>EDSS 1</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1E-3</v>
+      </c>
+      <c r="C3" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" t="str">
+        <f>Acaster!A4</f>
+        <v>EDSS 2</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-3.0000000000000001E-3</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" t="str">
+        <f>Acaster!A5</f>
+        <v>EDSS 3</v>
+      </c>
+      <c r="B5" s="4">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="C5" s="4">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" t="str">
+        <f>Acaster!A6</f>
+        <v>EDSS 4</v>
+      </c>
+      <c r="B6" s="4">
+        <v>-8.9999999999999993E-3</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="str">
+        <f>Acaster!A7</f>
+        <v>EDSS 5</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-0.02</v>
+      </c>
+      <c r="C7" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="str">
+        <f>Acaster!A8</f>
+        <v>EDSS 6</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-2.7E-2</v>
+      </c>
+      <c r="C8" s="4">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="str">
+        <f>Acaster!A9</f>
+        <v>EDSS 7</v>
+      </c>
+      <c r="B9" s="4">
+        <v>-5.2999999999999999E-2</v>
+      </c>
+      <c r="C9" s="4">
+        <v>1.0999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" t="str">
+        <f>Acaster!A10</f>
+        <v>EDSS 8</v>
+      </c>
+      <c r="B10" s="4">
+        <v>-0.107</v>
+      </c>
+      <c r="C10" s="4">
+        <v>2.1000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" t="str">
+        <f>Acaster!A11</f>
+        <v>EDSS 9</v>
+      </c>
+      <c r="B11" s="4">
+        <v>-0.14000000000000001</v>
+      </c>
+      <c r="C11" s="4">
+        <v>2.8000000000000001E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACE3D2A8E3060445845CB33F649944D9" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1dd74ed78a59e353fa0bdc00cb9d4ef2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a4e98822-f433-4c96-8830-5cb2d7491f7d" xmlns:ns3="adc125f1-7df9-46f4-a9a7-022dd426a2bb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="29b19980e720fd97176dcdbc89cda831" ns2:_="" ns3:_="">
     <xsd:import namespace="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
@@ -876,15 +1047,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -896,10 +1058,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F0B826-5EFE-4577-B049-981EAE9E4CA2}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1DBF9448-800E-4738-9636-5AD2000DD105}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -907,6 +1065,31 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{16F0B826-5EFE-4577-B049-981EAE9E4CA2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
+    <ds:schemaRef ds:uri="adc125f1-7df9-46f4-a9a7-022dd426a2bb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32834C50-F458-4BC1-999D-E35548F4265A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32834C50-F458-4BC1-999D-E35548F4265A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>